<commit_message>
feat(xiao-s3-tft): add portrait I2C, portrait EN-reset envs; fix meshnode pinout sheets
RiV_xiao-s3-tft-i2c and RiV_xiao-s3-tft-portrait-i2c swap the GPS for I2C on D5/D6.
RiV_xiao-s3-tft-portrait-en wires the LCD reset to EN, keeps I2C and SD, and
adds a receive-only GPS on D2. Touch rotation for it comes from touch_rotation.h
so each value builds without a full recompile. The meshnode ILI9488 pinout sheets
now say the LCD SDO stays unconnected.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/variants/esp32s3/diy/RiV_meshnode_s3_4in_joystick/RiV_meshnode_s3_4in_joystick_pinout.xlsx
+++ b/variants/esp32s3/diy/RiV_meshnode_s3_4in_joystick/RiV_meshnode_s3_4in_joystick_pinout.xlsx
@@ -440,9 +440,9 @@
   <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,7 +611,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>shared SPI bus</t>
+          <t>LoRa only. Do NOT connect the LCD SDO to this MISO</t>
         </is>
       </c>
     </row>
@@ -645,91 +645,91 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>ILI9341</t>
+          <t>ILI9488 4in; LCD SCK and SDI (MOSI) join the shared SCK and MOSI</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>I2C SDA / SCL</t>
+          <t>LCD_MISO/SDO</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>18 / 17</t>
+          <t>NOT CONNECTED</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>RTC PCF8563, BME280</t>
+          <t>leave unwired, it jams the radio</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>RTC_INT</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr"/>
+          <t>I2C SDA / SCL</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>18 / 17</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>RTC PCF8563, BME280</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>NEOPIXEL</t>
+          <t>RTC_INT</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>WS2812 x8</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>BUZZER</t>
+          <t>NEOPIXEL</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>WS2812 x8</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>BUZZER</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>BATTERY_ADC</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>LCD_MISO/SDO</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>not connected; it jams the radio</t>
-        </is>
-      </c>
+      <c r="C20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>